<commit_message>
add order cancel proceess
</commit_message>
<xml_diff>
--- a/scripts/test-data.xlsx
+++ b/scripts/test-data.xlsx
@@ -397,58 +397,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>email</v>
+        <v>user1@example.com</v>
       </c>
       <c r="B1" t="str">
-        <v>productlink</v>
+        <v>https://www.flipkart.com/apple-iphone-15-black-128-gb/p/itm6ac6485515ae4</v>
       </c>
       <c r="C1" t="str">
-        <v>name</v>
+        <v>krishan kumar</v>
       </c>
       <c r="D1" t="str">
-        <v>phone</v>
+        <v>9876543212</v>
       </c>
       <c r="E1" t="str">
-        <v>pincode</v>
+        <v>276135</v>
       </c>
       <c r="F1" t="str">
-        <v>addressline2</v>
+        <v>azamgarh</v>
       </c>
       <c r="G1" t="str">
-        <v>addressline2_1</v>
+        <v>village bibipur</v>
       </c>
       <c r="H1" t="str">
-        <v>city</v>
+        <v>azamgarh</v>
       </c>
       <c r="I1" t="str">
-        <v>state</v>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="J1" t="str">
-        <v>landmark</v>
+        <v>landmark didigoders</v>
       </c>
       <c r="K1" t="str">
-        <v>alternativephone</v>
+        <v>9876543211</v>
       </c>
       <c r="L1" t="str">
-        <v>password</v>
+        <v>pass123</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>user1@example.com</v>
+        <v>user2@example.com</v>
       </c>
       <c r="B2" t="str">
-        <v>https://www.flipkart.com/apple-iphone-15-black-128-gb/p/itm6ac6485515ae4</v>
+        <v>https://www.flipkart.com/samsung-galaxy-s23-fe-mint-128-gb/p/itmdd7c6e033924f</v>
       </c>
       <c r="C2" t="str">
-        <v>krishan kumar</v>
+        <v>bharti</v>
       </c>
       <c r="D2" t="str">
-        <v>9876543212</v>
+        <v>8765432198</v>
       </c>
       <c r="E2" t="str">
         <v>276135</v>
@@ -457,7 +457,7 @@
         <v>azamgarh</v>
       </c>
       <c r="G2" t="str">
-        <v>village bibipur</v>
+        <v>latgat</v>
       </c>
       <c r="H2" t="str">
         <v>azamgarh</v>
@@ -466,56 +466,18 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="J2" t="str">
-        <v>landmark didigoders</v>
+        <v>lata gath afdsf</v>
       </c>
       <c r="K2" t="str">
-        <v>9876543211</v>
+        <v>8765432112</v>
       </c>
       <c r="L2" t="str">
-        <v>pass123</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>user2@example.com</v>
-      </c>
-      <c r="B3" t="str">
-        <v>https://www.flipkart.com/samsung-galaxy-s23-fe-mint-128-gb/p/itmdd7c6e033924f</v>
-      </c>
-      <c r="C3" t="str">
-        <v>bharti</v>
-      </c>
-      <c r="D3" t="str">
-        <v>8765432198</v>
-      </c>
-      <c r="E3" t="str">
-        <v>276135</v>
-      </c>
-      <c r="F3" t="str">
-        <v>azamgarh</v>
-      </c>
-      <c r="G3" t="str">
-        <v>latgat</v>
-      </c>
-      <c r="H3" t="str">
-        <v>azamgarh</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Uttar Pradesh</v>
-      </c>
-      <c r="J3" t="str">
-        <v>lata gath afdsf</v>
-      </c>
-      <c r="K3" t="str">
-        <v>8765432112</v>
-      </c>
-      <c r="L3" t="str">
         <v>pass456</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>